<commit_message>
Otm Guncelleme: (2026-09-24 12:41:27)
</commit_message>
<xml_diff>
--- a/bugun_oranlar.xlsx
+++ b/bugun_oranlar.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H97"/>
+  <dimension ref="A1:H95"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -461,28 +461,28 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>51 dk içinde</t>
+          <t>21:00</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Oud-Heverlee Leuven (K) vs AS Roma (K)</t>
+          <t>Belçika U21 vs Belarus U21</t>
         </is>
       </c>
       <c r="C2" t="n">
-        <v>4.75</v>
+        <v>1.2</v>
       </c>
       <c r="D2" t="n">
-        <v>4</v>
+        <v>5.5</v>
       </c>
       <c r="E2" t="n">
-        <v>1.55</v>
+        <v>12</v>
       </c>
       <c r="F2" t="n">
-        <v>1.55</v>
+        <v>1.58</v>
       </c>
       <c r="G2" t="n">
-        <v>2.23</v>
+        <v>2.2</v>
       </c>
       <c r="H2" t="inlineStr">
         <is>
@@ -493,28 +493,28 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>51 dk içinde</t>
+          <t>21:30</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Servette Chenois (K) vs Lyon (K)</t>
+          <t>San Marino U21 vs Kosovo U21</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>46</v>
+        <v>36</v>
       </c>
       <c r="D3" t="n">
-        <v>19</v>
+        <v>15</v>
       </c>
       <c r="E3" t="n">
-        <v>1.08</v>
+        <v>1.12</v>
       </c>
       <c r="F3" t="n">
-        <v>1.08</v>
+        <v>1.12</v>
       </c>
       <c r="G3" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="H3" t="inlineStr">
         <is>
@@ -525,28 +525,28 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>22:00</t>
+          <t>21:45</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Barcelona (K) vs Paris FC (K)</t>
+          <t>Portekiz vs Galler</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>17</v>
+        <v>1.18</v>
       </c>
       <c r="D4" t="n">
-        <v>36</v>
+        <v>6.5</v>
       </c>
       <c r="E4" t="n">
-        <v>1.08</v>
+        <v>13.25</v>
       </c>
       <c r="F4" t="n">
-        <v>1.08</v>
+        <v>1.41</v>
       </c>
       <c r="G4" t="n">
-        <v>6.5</v>
+        <v>2.68</v>
       </c>
       <c r="H4" t="inlineStr">
         <is>
@@ -557,28 +557,28 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>22:00</t>
+          <t>21:45</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Chelsea (K) vs Austria Vienna (K)</t>
+          <t>Norveç vs Danimarka</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>15</v>
+        <v>1.81</v>
       </c>
       <c r="D5" t="n">
-        <v>46</v>
+        <v>3.8</v>
       </c>
       <c r="E5" t="n">
-        <v>1.18</v>
+        <v>3.8</v>
       </c>
       <c r="F5" t="n">
-        <v>1.18</v>
+        <v>1.62</v>
       </c>
       <c r="G5" t="n">
-        <v>4.2</v>
+        <v>2.25</v>
       </c>
       <c r="H5" t="inlineStr">
         <is>
@@ -589,28 +589,28 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>6 dk içinde</t>
+          <t>21:45</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Breidablik Kopavogur (K) vs Czarni Sosnowiec (K)</t>
+          <t>Sırbistan vs Yunanistan</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>2.2</v>
+        <v>2.73</v>
       </c>
       <c r="D6" t="n">
-        <v>3.6</v>
+        <v>3.2</v>
       </c>
       <c r="E6" t="n">
         <v>2.6</v>
       </c>
       <c r="F6" t="n">
-        <v>1.47</v>
+        <v>2.22</v>
       </c>
       <c r="G6" t="n">
-        <v>2.4</v>
+        <v>1.62</v>
       </c>
       <c r="H6" t="inlineStr">
         <is>
@@ -621,28 +621,28 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>6 dk içinde</t>
+          <t>21:45</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Sparta Prague (K) vs Farul Constanta (K)</t>
+          <t>Hollanda vs Almanya</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>1.05</v>
+        <v>2.5</v>
       </c>
       <c r="D7" t="n">
-        <v>9</v>
+        <v>3.8</v>
       </c>
       <c r="E7" t="n">
-        <v>21</v>
+        <v>2.45</v>
       </c>
       <c r="F7" t="n">
-        <v>1.27</v>
+        <v>1.43</v>
       </c>
       <c r="G7" t="n">
-        <v>3.3</v>
+        <v>2.6</v>
       </c>
       <c r="H7" t="inlineStr">
         <is>
@@ -653,28 +653,28 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>6 dk içinde</t>
+          <t>21:45</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Brondby (K) vs Sporting (K)</t>
+          <t>Avusturya vs İsrail</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>2.6</v>
+        <v>1.43</v>
       </c>
       <c r="D8" t="n">
-        <v>3.3</v>
+        <v>4.5</v>
       </c>
       <c r="E8" t="n">
-        <v>2.27</v>
+        <v>6</v>
       </c>
       <c r="F8" t="n">
-        <v>1.71</v>
+        <v>1.51</v>
       </c>
       <c r="G8" t="n">
-        <v>1.98</v>
+        <v>2.45</v>
       </c>
       <c r="H8" t="inlineStr">
         <is>
@@ -685,28 +685,28 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>51 dk içinde</t>
+          <t>21:45</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>St. Polten (K) vs Malmo FF (K)</t>
+          <t>Kosova vs İrlanda</t>
         </is>
       </c>
       <c r="C9" t="n">
+        <v>2.4</v>
+      </c>
+      <c r="D9" t="n">
         <v>3.2</v>
       </c>
-      <c r="D9" t="n">
-        <v>3.6</v>
-      </c>
       <c r="E9" t="n">
-        <v>1.87</v>
+        <v>3</v>
       </c>
       <c r="F9" t="n">
-        <v>1.6</v>
+        <v>2.3</v>
       </c>
       <c r="G9" t="n">
-        <v>2.16</v>
+        <v>1.58</v>
       </c>
       <c r="H9" t="inlineStr">
         <is>
@@ -717,28 +717,28 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>20:00</t>
+          <t>21:45</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Feyenoord (K) vs Valerenga (K)</t>
+          <t>Lihtenştayn vs Litvanya</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>2.6</v>
+        <v>10</v>
       </c>
       <c r="D10" t="n">
-        <v>3.6</v>
+        <v>4.5</v>
       </c>
       <c r="E10" t="n">
-        <v>2.2</v>
+        <v>1.3</v>
       </c>
       <c r="F10" t="n">
-        <v>1.47</v>
+        <v>2.05</v>
       </c>
       <c r="G10" t="n">
-        <v>2.39</v>
+        <v>1.68</v>
       </c>
       <c r="H10" t="inlineStr">
         <is>
@@ -749,28 +749,28 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>20:00</t>
+          <t>19:00</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>PSV (K) vs Fortuna Hjorring (K)</t>
+          <t>Andorra vs Malta</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>1.37</v>
+        <v>3.28</v>
       </c>
       <c r="D11" t="n">
-        <v>4.33</v>
+        <v>2.8</v>
       </c>
       <c r="E11" t="n">
-        <v>6</v>
+        <v>2.4</v>
       </c>
       <c r="F11" t="n">
-        <v>1.53</v>
+        <v>3</v>
       </c>
       <c r="G11" t="n">
-        <v>2.33</v>
+        <v>1.33</v>
       </c>
       <c r="H11" t="inlineStr">
         <is>
@@ -781,28 +781,28 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>20:00</t>
+          <t>21:45</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Hammarby IF (K) vs Rangers (K)</t>
+          <t>Boldmere St. Michaels (W) vs Sutton Coldfield (W)</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>1.3</v>
+        <v>1.07</v>
       </c>
       <c r="D12" t="n">
-        <v>4.75</v>
+        <v>8</v>
       </c>
       <c r="E12" t="n">
-        <v>6.5</v>
+        <v>13.25</v>
       </c>
       <c r="F12" t="n">
-        <v>1.43</v>
+        <v>1.72</v>
       </c>
       <c r="G12" t="n">
-        <v>2.59</v>
+        <v>2</v>
       </c>
       <c r="H12" t="inlineStr">
         <is>
@@ -813,28 +813,28 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>20:00</t>
+          <t>21:45</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Wolfsburg (K) vs Sturm Graz (K)</t>
+          <t>Stade Caen vs Rouen</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>1.006</v>
+        <v>2.54</v>
       </c>
       <c r="D13" t="n">
-        <v>15</v>
+        <v>3.2</v>
       </c>
       <c r="E13" t="n">
-        <v>36</v>
+        <v>2.4</v>
       </c>
       <c r="F13" t="n">
-        <v>1.12</v>
+        <v>1.84</v>
       </c>
       <c r="G13" t="n">
-        <v>5</v>
+        <v>1.83</v>
       </c>
       <c r="H13" t="inlineStr">
         <is>
@@ -845,28 +845,28 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>20:30</t>
+          <t>16:25</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Ajax (K) vs Aktobe (K)</t>
+          <t>Al Dhaid U21 vs Shabab Al Ahli Dubai U21</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>1.01</v>
+        <v>3.4</v>
       </c>
       <c r="D14" t="n">
-        <v>13.25</v>
+        <v>3.8</v>
       </c>
       <c r="E14" t="n">
-        <v>29</v>
+        <v>1.66</v>
       </c>
       <c r="F14" t="n">
-        <v>1.11</v>
+        <v>1.35</v>
       </c>
       <c r="G14" t="n">
-        <v>5.5</v>
+        <v>2.8</v>
       </c>
       <c r="H14" t="inlineStr">
         <is>
@@ -877,28 +877,28 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>21:00</t>
+          <t>16:30</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Hearts (K) vs Real Sociedad (K)</t>
+          <t>Al Jazira SC U21 vs Al Orooba U21</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>6.5</v>
+        <v>1.28</v>
       </c>
       <c r="D15" t="n">
         <v>4.75</v>
       </c>
       <c r="E15" t="n">
+        <v>6.5</v>
+      </c>
+      <c r="F15" t="n">
         <v>1.33</v>
       </c>
-      <c r="F15" t="n">
-        <v>1.4</v>
-      </c>
       <c r="G15" t="n">
-        <v>2.7</v>
+        <v>2.8</v>
       </c>
       <c r="H15" t="inlineStr">
         <is>
@@ -914,23 +914,23 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Liverpool (K) vs Sunderland (W)</t>
+          <t>Portuguesa de Desportos U20 vs Ponte Preta SP U20</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>1.2</v>
+        <v>1.64</v>
       </c>
       <c r="D16" t="n">
-        <v>5.5</v>
+        <v>3.7</v>
       </c>
       <c r="E16" t="n">
-        <v>9.5</v>
+        <v>4</v>
       </c>
       <c r="F16" t="n">
-        <v>1.37</v>
+        <v>1.62</v>
       </c>
       <c r="G16" t="n">
-        <v>2.7</v>
+        <v>2.12</v>
       </c>
       <c r="H16" t="inlineStr">
         <is>
@@ -941,28 +941,28 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>21:00</t>
+          <t>14:00</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Everton (K) vs Birmingham (K)</t>
+          <t>Viborg U19 vs Brondby U19</t>
         </is>
       </c>
       <c r="C17" t="n">
-        <v>1.87</v>
+        <v>2.45</v>
       </c>
       <c r="D17" t="n">
-        <v>3.3</v>
+        <v>3.6</v>
       </c>
       <c r="E17" t="n">
-        <v>3.4</v>
+        <v>2.34</v>
       </c>
       <c r="F17" t="n">
-        <v>1.87</v>
+        <v>1.5</v>
       </c>
       <c r="G17" t="n">
-        <v>1.79</v>
+        <v>2.33</v>
       </c>
       <c r="H17" t="inlineStr">
         <is>
@@ -973,28 +973,28 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>21:00</t>
+          <t>16:00</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Tottenham (K) vs West Ham (K)</t>
+          <t>Hartberg vs Kapfenberg</t>
         </is>
       </c>
       <c r="C18" t="n">
-        <v>1.25</v>
+        <v>1.43</v>
       </c>
       <c r="D18" t="n">
-        <v>4.75</v>
+        <v>4.33</v>
       </c>
       <c r="E18" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="F18" t="n">
-        <v>1.47</v>
+        <v>1.43</v>
       </c>
       <c r="G18" t="n">
-        <v>2.34</v>
+        <v>2.6</v>
       </c>
       <c r="H18" t="inlineStr">
         <is>
@@ -1005,28 +1005,28 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>21:00</t>
+          <t>19:30</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Nottingham Forest (W) vs Aston Villa (K)</t>
+          <t>SF Siegen 1899 vs Borussia Monchengladbach</t>
         </is>
       </c>
       <c r="C19" t="n">
-        <v>3.7</v>
+        <v>31</v>
       </c>
       <c r="D19" t="n">
-        <v>3.7</v>
+        <v>13.25</v>
       </c>
       <c r="E19" t="n">
-        <v>1.71</v>
+        <v>1.02</v>
       </c>
       <c r="F19" t="n">
-        <v>1.55</v>
+        <v>1.14</v>
       </c>
       <c r="G19" t="n">
-        <v>2.22</v>
+        <v>4.5</v>
       </c>
       <c r="H19" t="inlineStr">
         <is>
@@ -1037,28 +1037,28 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>21:00</t>
+          <t>20:00</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Manchester United (K) vs Sheffield United FC (W)</t>
+          <t>SC Rot-Weiss Oberhausen vs Schalke 04</t>
         </is>
       </c>
       <c r="C20" t="n">
-        <v>1.03</v>
+        <v>7</v>
       </c>
       <c r="D20" t="n">
-        <v>9.5</v>
+        <v>5</v>
       </c>
       <c r="E20" t="n">
-        <v>23</v>
+        <v>1.28</v>
       </c>
       <c r="F20" t="n">
-        <v>1.22</v>
+        <v>1.25</v>
       </c>
       <c r="G20" t="n">
-        <v>3.3</v>
+        <v>3.5</v>
       </c>
       <c r="H20" t="inlineStr">
         <is>
@@ -1069,28 +1069,28 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>21:00</t>
+          <t>14:00</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Crystal Palace (K) vs Watford (W)</t>
+          <t>Hollanda U19 vs Belçika U19</t>
         </is>
       </c>
       <c r="C21" t="n">
-        <v>1.18</v>
+        <v>2.09</v>
       </c>
       <c r="D21" t="n">
-        <v>5.5</v>
+        <v>3.5</v>
       </c>
       <c r="E21" t="n">
-        <v>9</v>
+        <v>2.73</v>
       </c>
       <c r="F21" t="n">
-        <v>1.28</v>
+        <v>1.5</v>
       </c>
       <c r="G21" t="n">
-        <v>3.05</v>
+        <v>2.37</v>
       </c>
       <c r="H21" t="inlineStr">
         <is>
@@ -1101,28 +1101,28 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>21:30</t>
+          <t>17:00</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Leicester (K) vs London City Lionesses (K)</t>
+          <t>Sırbistan U19 vs Bulgaristan U19</t>
         </is>
       </c>
       <c r="C22" t="n">
-        <v>9.5</v>
+        <v>1.98</v>
       </c>
       <c r="D22" t="n">
-        <v>5.5</v>
+        <v>3.3</v>
       </c>
       <c r="E22" t="n">
-        <v>1.18</v>
+        <v>3.1</v>
       </c>
       <c r="F22" t="n">
-        <v>1.33</v>
+        <v>1.76</v>
       </c>
       <c r="G22" t="n">
-        <v>2.8</v>
+        <v>1.92</v>
       </c>
       <c r="H22" t="inlineStr">
         <is>
@@ -1133,28 +1133,28 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>21:45</t>
+          <t>17:00</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Brighton (K) vs Charlton (K)</t>
+          <t>Romanya U19 vs Macaristan U19</t>
         </is>
       </c>
       <c r="C23" t="n">
-        <v>1.2</v>
+        <v>2.16</v>
       </c>
       <c r="D23" t="n">
-        <v>5</v>
+        <v>3.4</v>
       </c>
       <c r="E23" t="n">
-        <v>8.5</v>
+        <v>2.73</v>
       </c>
       <c r="F23" t="n">
-        <v>1.4</v>
+        <v>1.66</v>
       </c>
       <c r="G23" t="n">
-        <v>2.59</v>
+        <v>2.06</v>
       </c>
       <c r="H23" t="inlineStr">
         <is>
@@ -1165,28 +1165,28 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>21:45</t>
+          <t>30 dk içinde</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Kingstonian vs Bedfont</t>
+          <t>Japonya vs Uruguay</t>
         </is>
       </c>
       <c r="C24" t="n">
-        <v>1.85</v>
+        <v>1.64</v>
       </c>
       <c r="D24" t="n">
-        <v>3.6</v>
+        <v>3.8</v>
       </c>
       <c r="E24" t="n">
-        <v>3.2</v>
+        <v>4.75</v>
       </c>
       <c r="F24" t="n">
-        <v>1.51</v>
+        <v>1.87</v>
       </c>
       <c r="G24" t="n">
-        <v>2.34</v>
+        <v>1.83</v>
       </c>
       <c r="H24" t="inlineStr">
         <is>
@@ -1197,28 +1197,28 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>21:30</t>
+          <t>14:00</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Sevenoaks Town vs Eastbourne Town</t>
+          <t>Kore Cumhuriyeti vs Ekvador</t>
         </is>
       </c>
       <c r="C25" t="n">
-        <v>2.04</v>
+        <v>2.18</v>
       </c>
       <c r="D25" t="n">
-        <v>3.5</v>
+        <v>3.2</v>
       </c>
       <c r="E25" t="n">
-        <v>2.8</v>
+        <v>3.15</v>
       </c>
       <c r="F25" t="n">
-        <v>1.57</v>
+        <v>2.12</v>
       </c>
       <c r="G25" t="n">
-        <v>2.22</v>
+        <v>1.66</v>
       </c>
       <c r="H25" t="inlineStr">
         <is>
@@ -1229,28 +1229,28 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>21:00</t>
+          <t>14:35</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Boreham Wood vs Everton U21</t>
+          <t>Çin vs Maldives</t>
         </is>
       </c>
       <c r="C26" t="n">
-        <v>1.18</v>
+        <v>1.02</v>
       </c>
       <c r="D26" t="n">
-        <v>6</v>
+        <v>17</v>
       </c>
       <c r="E26" t="n">
-        <v>10</v>
+        <v>46</v>
       </c>
       <c r="F26" t="n">
-        <v>1.28</v>
+        <v>1.12</v>
       </c>
       <c r="G26" t="n">
-        <v>3.2</v>
+        <v>5</v>
       </c>
       <c r="H26" t="inlineStr">
         <is>
@@ -1261,28 +1261,28 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>21:45</t>
+          <t>17:00</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Guisborough Town vs Ashington</t>
+          <t>Özbekistan vs Iran</t>
         </is>
       </c>
       <c r="C27" t="n">
-        <v>1.83</v>
+        <v>2.77</v>
       </c>
       <c r="D27" t="n">
-        <v>3.5</v>
+        <v>3</v>
       </c>
       <c r="E27" t="n">
-        <v>3.4</v>
+        <v>2.59</v>
       </c>
       <c r="F27" t="n">
-        <v>1.66</v>
+        <v>2.45</v>
       </c>
       <c r="G27" t="n">
-        <v>2.03</v>
+        <v>1.47</v>
       </c>
       <c r="H27" t="inlineStr">
         <is>
@@ -1293,28 +1293,28 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>21:45</t>
+          <t>22:00</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Shifnal Town vs Nantwich Town</t>
+          <t>Atletico Rojiblanco vs CD Cuenca Juniors</t>
         </is>
       </c>
       <c r="C28" t="n">
-        <v>2.5</v>
+        <v>1.99</v>
       </c>
       <c r="D28" t="n">
-        <v>3.5</v>
+        <v>3</v>
       </c>
       <c r="E28" t="n">
-        <v>2.27</v>
+        <v>3.6</v>
       </c>
       <c r="F28" t="n">
-        <v>1.55</v>
+        <v>2.45</v>
       </c>
       <c r="G28" t="n">
-        <v>2.25</v>
+        <v>1.45</v>
       </c>
       <c r="H28" t="inlineStr">
         <is>
@@ -1325,28 +1325,28 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>21:45</t>
+          <t>23:30</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Lower Breck vs Atherton Collieries</t>
+          <t>Indepiendente Juniors vs Vinotinto Ecuador</t>
         </is>
       </c>
       <c r="C29" t="n">
         <v>2.16</v>
       </c>
       <c r="D29" t="n">
-        <v>3.5</v>
+        <v>3</v>
       </c>
       <c r="E29" t="n">
-        <v>2.63</v>
+        <v>3.1</v>
       </c>
       <c r="F29" t="n">
-        <v>1.58</v>
+        <v>2.36</v>
       </c>
       <c r="G29" t="n">
-        <v>2.18</v>
+        <v>1.51</v>
       </c>
       <c r="H29" t="inlineStr">
         <is>
@@ -1357,28 +1357,28 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>21:45</t>
+          <t>17:00</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>London Lions vs Biggleswade</t>
+          <t>FC Elva vs JK Tallinna Kalev</t>
         </is>
       </c>
       <c r="C30" t="n">
-        <v>4.2</v>
+        <v>2.63</v>
       </c>
       <c r="D30" t="n">
-        <v>4</v>
+        <v>3.6</v>
       </c>
       <c r="E30" t="n">
-        <v>1.58</v>
+        <v>2.2</v>
       </c>
       <c r="F30" t="n">
-        <v>1.41</v>
+        <v>1.51</v>
       </c>
       <c r="G30" t="n">
-        <v>2.63</v>
+        <v>2.35</v>
       </c>
       <c r="H30" t="inlineStr">
         <is>
@@ -1389,28 +1389,28 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>21:00</t>
+          <t>18:00</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Saguntino vs Navalcarnero</t>
+          <t>FAR Rabat vs Raja Casablanca</t>
         </is>
       </c>
       <c r="C31" t="n">
-        <v>2.6</v>
+        <v>2.2</v>
       </c>
       <c r="D31" t="n">
-        <v>3</v>
+        <v>2.35</v>
       </c>
       <c r="E31" t="n">
-        <v>2.45</v>
+        <v>3.5</v>
       </c>
       <c r="F31" t="n">
-        <v>2.26</v>
+        <v>2.35</v>
       </c>
       <c r="G31" t="n">
-        <v>1.55</v>
+        <v>1.51</v>
       </c>
       <c r="H31" t="inlineStr">
         <is>
@@ -1421,28 +1421,28 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>22:00</t>
+          <t>23:00</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Sant Andreu Barcelona vs Real Madrid B</t>
+          <t>Amal Tiznit vs Ittihad Riadhi de Tanger</t>
         </is>
       </c>
       <c r="C32" t="n">
-        <v>3</v>
+        <v>3.05</v>
       </c>
       <c r="D32" t="n">
-        <v>3.2</v>
+        <v>2.77</v>
       </c>
       <c r="E32" t="n">
-        <v>2.11</v>
+        <v>2.31</v>
       </c>
       <c r="F32" t="n">
-        <v>2.01</v>
+        <v>2.9</v>
       </c>
       <c r="G32" t="n">
-        <v>1.7</v>
+        <v>1.35</v>
       </c>
       <c r="H32" t="inlineStr">
         <is>
@@ -1453,28 +1453,28 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>21:00</t>
+          <t>18:15</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>VV Zwaluwen Vlaardingen vs VPV Purmersteijn</t>
+          <t>JyTy vs Abo CF</t>
         </is>
       </c>
       <c r="C33" t="n">
-        <v>2.33</v>
+        <v>1.51</v>
       </c>
       <c r="D33" t="n">
-        <v>3.7</v>
+        <v>4.2</v>
       </c>
       <c r="E33" t="n">
-        <v>2.4</v>
+        <v>4.33</v>
       </c>
       <c r="F33" t="n">
-        <v>1.43</v>
+        <v>1.33</v>
       </c>
       <c r="G33" t="n">
-        <v>2.6</v>
+        <v>2.8</v>
       </c>
       <c r="H33" t="inlineStr">
         <is>
@@ -1485,28 +1485,28 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>21:00</t>
+          <t>19:00</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Tot Ons Genoegen Berkel vs ROHDA Raalte</t>
+          <t>Fc Kontu vs Lps</t>
         </is>
       </c>
       <c r="C34" t="n">
-        <v>3.5</v>
+        <v>4</v>
       </c>
       <c r="D34" t="n">
-        <v>4.25</v>
+        <v>4.5</v>
       </c>
       <c r="E34" t="n">
-        <v>1.68</v>
+        <v>1.55</v>
       </c>
       <c r="F34" t="n">
-        <v>1.22</v>
+        <v>1.18</v>
       </c>
       <c r="G34" t="n">
-        <v>3.7</v>
+        <v>4</v>
       </c>
       <c r="H34" t="inlineStr">
         <is>
@@ -1517,28 +1517,28 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>21:00</t>
+          <t>19:00</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>JOS/Watergraafsmeer vs Tielse EC</t>
+          <t>LAUTP/2 vs Kultsu</t>
         </is>
       </c>
       <c r="C35" t="n">
-        <v>4.33</v>
+        <v>19</v>
       </c>
       <c r="D35" t="n">
-        <v>4.5</v>
+        <v>10</v>
       </c>
       <c r="E35" t="n">
-        <v>1.51</v>
+        <v>1.03</v>
       </c>
       <c r="F35" t="n">
-        <v>1.25</v>
+        <v>1.11</v>
       </c>
       <c r="G35" t="n">
-        <v>3.4</v>
+        <v>5.5</v>
       </c>
       <c r="H35" t="inlineStr">
         <is>
@@ -1549,28 +1549,28 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>21:00</t>
+          <t>19:00</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>VV Sparta Nijkerk vs UDI '19</t>
+          <t>Eif/Akademi vs HooGee</t>
         </is>
       </c>
       <c r="C36" t="n">
-        <v>2.08</v>
+        <v>1.41</v>
       </c>
       <c r="D36" t="n">
-        <v>3.8</v>
+        <v>4.75</v>
       </c>
       <c r="E36" t="n">
-        <v>2.73</v>
+        <v>4.5</v>
       </c>
       <c r="F36" t="n">
-        <v>1.32</v>
+        <v>1.14</v>
       </c>
       <c r="G36" t="n">
-        <v>3.05</v>
+        <v>5</v>
       </c>
       <c r="H36" t="inlineStr">
         <is>
@@ -1581,28 +1581,28 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>21:00</t>
+          <t>20:00</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>IJsselmeervogels vs VV Gemert</t>
+          <t>PPJ/Lauttasaari vs Pakkalan Palloseura</t>
         </is>
       </c>
       <c r="C37" t="n">
-        <v>1.28</v>
+        <v>1.05</v>
       </c>
       <c r="D37" t="n">
+        <v>9.5</v>
+      </c>
+      <c r="E37" t="n">
+        <v>15</v>
+      </c>
+      <c r="F37" t="n">
+        <v>1.14</v>
+      </c>
+      <c r="G37" t="n">
         <v>5</v>
-      </c>
-      <c r="E37" t="n">
-        <v>8</v>
-      </c>
-      <c r="F37" t="n">
-        <v>1.47</v>
-      </c>
-      <c r="G37" t="n">
-        <v>2.4</v>
       </c>
       <c r="H37" t="inlineStr">
         <is>
@@ -1613,28 +1613,28 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>21:00</t>
+          <t>20:00</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>CA Sarmiento Reserves vs Atletico Rafaela Reserves</t>
+          <t>Fish United vs Saaksjaerven Loiske</t>
         </is>
       </c>
       <c r="C38" t="n">
-        <v>2.25</v>
+        <v>2.58</v>
       </c>
       <c r="D38" t="n">
-        <v>3.1</v>
+        <v>3.8</v>
       </c>
       <c r="E38" t="n">
-        <v>2.8</v>
+        <v>2.12</v>
       </c>
       <c r="F38" t="n">
-        <v>2.12</v>
+        <v>1.27</v>
       </c>
       <c r="G38" t="n">
-        <v>1.64</v>
+        <v>3.15</v>
       </c>
       <c r="H38" t="inlineStr">
         <is>
@@ -1645,28 +1645,28 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>21:00</t>
+          <t>20:30</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Gimnasia La Plata Reserves vs Estudiantes La Plata Reserves</t>
+          <t>MPS vs Poxyt</t>
         </is>
       </c>
       <c r="C39" t="n">
+        <v>2.27</v>
+      </c>
+      <c r="D39" t="n">
+        <v>3.7</v>
+      </c>
+      <c r="E39" t="n">
         <v>2.45</v>
       </c>
-      <c r="D39" t="n">
-        <v>2.9</v>
-      </c>
-      <c r="E39" t="n">
-        <v>2.63</v>
-      </c>
       <c r="F39" t="n">
-        <v>2.3</v>
+        <v>1.35</v>
       </c>
       <c r="G39" t="n">
-        <v>1.53</v>
+        <v>2.73</v>
       </c>
       <c r="H39" t="inlineStr">
         <is>
@@ -1677,28 +1677,28 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>21:00</t>
+          <t>18:00</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>CA Aldosivi Reserves vs Quilmes Reserves</t>
+          <t>NK Koprivnica vs NK Uskok</t>
         </is>
       </c>
       <c r="C40" t="n">
-        <v>2.58</v>
+        <v>2.45</v>
       </c>
       <c r="D40" t="n">
-        <v>3.1</v>
+        <v>3.5</v>
       </c>
       <c r="E40" t="n">
-        <v>2.45</v>
+        <v>2.31</v>
       </c>
       <c r="F40" t="n">
-        <v>2.12</v>
+        <v>1.53</v>
       </c>
       <c r="G40" t="n">
-        <v>1.62</v>
+        <v>2.26</v>
       </c>
       <c r="H40" t="inlineStr">
         <is>
@@ -1709,28 +1709,28 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>21:00</t>
+          <t>53 dk içinde</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Defensa Y Justicia Reserves vs Tigre Reserves</t>
+          <t>Rebels Fc vs Roots</t>
         </is>
       </c>
       <c r="C41" t="n">
-        <v>1.72</v>
+        <v>2.39</v>
       </c>
       <c r="D41" t="n">
-        <v>3.4</v>
+        <v>3.1</v>
       </c>
       <c r="E41" t="n">
-        <v>4</v>
+        <v>2.6</v>
       </c>
       <c r="F41" t="n">
-        <v>1.87</v>
+        <v>2.04</v>
       </c>
       <c r="G41" t="n">
-        <v>1.8</v>
+        <v>1.66</v>
       </c>
       <c r="H41" t="inlineStr">
         <is>
@@ -1741,28 +1741,28 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>23:00</t>
+          <t>19:00</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>Lanus Reserves vs Banfield Reserves</t>
+          <t>FC Jerusalem vs Maccabi Yavne</t>
         </is>
       </c>
       <c r="C42" t="n">
-        <v>1.71</v>
+        <v>2.09</v>
       </c>
       <c r="D42" t="n">
-        <v>3.7</v>
+        <v>3.3</v>
       </c>
       <c r="E42" t="n">
-        <v>3.7</v>
+        <v>2.9</v>
       </c>
       <c r="F42" t="n">
-        <v>1.53</v>
+        <v>1.8</v>
       </c>
       <c r="G42" t="n">
-        <v>2.27</v>
+        <v>1.87</v>
       </c>
       <c r="H42" t="inlineStr">
         <is>
@@ -1773,28 +1773,28 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>20:00</t>
+          <t>19:45</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>CA Atlas Reserves vs Argentino de Rosario Reserves</t>
+          <t>Hapoel Tzafririm Holon vs Kfar Saba 1928</t>
         </is>
       </c>
       <c r="C43" t="n">
-        <v>2.03</v>
+        <v>2.9</v>
       </c>
       <c r="D43" t="n">
-        <v>3.4</v>
+        <v>3.15</v>
       </c>
       <c r="E43" t="n">
-        <v>2.9</v>
+        <v>2.15</v>
       </c>
       <c r="F43" t="n">
-        <v>1.64</v>
+        <v>1.99</v>
       </c>
       <c r="G43" t="n">
-        <v>2.05</v>
+        <v>1.71</v>
       </c>
       <c r="H43" t="inlineStr">
         <is>
@@ -1805,28 +1805,28 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>20:30</t>
+          <t>20:15</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>Canuelas FC Reserves vs Leones de Rosario Reserves</t>
+          <t>Hapoel Hadera vs Maccabi Ashdod</t>
         </is>
       </c>
       <c r="C44" t="n">
-        <v>1.94</v>
+        <v>1.76</v>
       </c>
       <c r="D44" t="n">
-        <v>3.3</v>
+        <v>3.4</v>
       </c>
       <c r="E44" t="n">
-        <v>3.2</v>
+        <v>3.7</v>
       </c>
       <c r="F44" t="n">
-        <v>1.84</v>
+        <v>1.79</v>
       </c>
       <c r="G44" t="n">
-        <v>1.85</v>
+        <v>1.87</v>
       </c>
       <c r="H44" t="inlineStr">
         <is>
@@ -1837,28 +1837,28 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>21:00</t>
+          <t>19:00</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>Lanus (K) vs River Plate (K)</t>
+          <t>Ironi Modiin vs MS Ashdod</t>
         </is>
       </c>
       <c r="C45" t="n">
-        <v>4.75</v>
+        <v>6</v>
       </c>
       <c r="D45" t="n">
-        <v>3.4</v>
+        <v>4.2</v>
       </c>
       <c r="E45" t="n">
-        <v>1.62</v>
+        <v>1.4</v>
       </c>
       <c r="F45" t="n">
-        <v>2.04</v>
+        <v>1.7</v>
       </c>
       <c r="G45" t="n">
-        <v>1.66</v>
+        <v>2.03</v>
       </c>
       <c r="H45" t="inlineStr">
         <is>
@@ -1869,28 +1869,28 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>3 dk içinde</t>
+          <t>19:00</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>Tristan Suarez Reserves vs Defensores De Belgrano</t>
+          <t>Maccabi Herzliya vs Kiryat Yam</t>
         </is>
       </c>
       <c r="C46" t="n">
-        <v>2.08</v>
+        <v>2.54</v>
       </c>
       <c r="D46" t="n">
-        <v>3</v>
+        <v>3.3</v>
       </c>
       <c r="E46" t="n">
-        <v>3.2</v>
+        <v>2.37</v>
       </c>
       <c r="F46" t="n">
-        <v>2.3</v>
+        <v>1.76</v>
       </c>
       <c r="G46" t="n">
-        <v>1.55</v>
+        <v>1.92</v>
       </c>
       <c r="H46" t="inlineStr">
         <is>
@@ -1901,28 +1901,28 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>22:30</t>
+          <t>19:00</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>Sportivo Desamparados vs Sportivo Rivadavia San Juan</t>
+          <t>Hapoel Ironi Rishon Lezion vs Maccabi Ahi Nazareth FC</t>
         </is>
       </c>
       <c r="C47" t="n">
-        <v>1.83</v>
+        <v>1.6</v>
       </c>
       <c r="D47" t="n">
-        <v>3.5</v>
+        <v>3.8</v>
       </c>
       <c r="E47" t="n">
-        <v>3.4</v>
+        <v>4.33</v>
       </c>
       <c r="F47" t="n">
-        <v>1.64</v>
+        <v>1.58</v>
       </c>
       <c r="G47" t="n">
-        <v>2.01</v>
+        <v>2.2</v>
       </c>
       <c r="H47" t="inlineStr">
         <is>
@@ -1933,28 +1933,28 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>22:30</t>
+          <t>19:00</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>Sarmiento de Zonda vs CA Union Villa Krause</t>
+          <t>Hapoel Akko FC vs Hapoel Afula</t>
         </is>
       </c>
       <c r="C48" t="n">
         <v>4.25</v>
       </c>
       <c r="D48" t="n">
-        <v>3.6</v>
+        <v>3.7</v>
       </c>
       <c r="E48" t="n">
-        <v>1.62</v>
+        <v>1.64</v>
       </c>
       <c r="F48" t="n">
-        <v>1.68</v>
+        <v>1.66</v>
       </c>
       <c r="G48" t="n">
-        <v>1.97</v>
+        <v>2.06</v>
       </c>
       <c r="H48" t="inlineStr">
         <is>
@@ -1965,28 +1965,28 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>21:00</t>
+          <t>14:45</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>Suudi Arabistan vs Kuveyt</t>
+          <t>Maccabi Kiryat Ata Bialik vs Hapoel Ihud Bnei Jatt</t>
         </is>
       </c>
       <c r="C49" t="n">
-        <v>1.33</v>
+        <v>1.18</v>
       </c>
       <c r="D49" t="n">
-        <v>4.5</v>
+        <v>5.5</v>
       </c>
       <c r="E49" t="n">
-        <v>7.5</v>
+        <v>10</v>
       </c>
       <c r="F49" t="n">
-        <v>1.68</v>
+        <v>1.43</v>
       </c>
       <c r="G49" t="n">
-        <v>2.06</v>
+        <v>2.02</v>
       </c>
       <c r="H49" t="inlineStr">
         <is>
@@ -1997,28 +1997,28 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>20:00</t>
+          <t>16:30</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>SV Gerasdorf Stammersdorf vs Sportunion Mauer</t>
+          <t>Maccabi Nujeidat Ahmed vs Hapoel Ironi Arraba</t>
         </is>
       </c>
       <c r="C50" t="n">
-        <v>7</v>
+        <v>1.87</v>
       </c>
       <c r="D50" t="n">
-        <v>4.5</v>
+        <v>3.5</v>
       </c>
       <c r="E50" t="n">
-        <v>1.3</v>
+        <v>3.3</v>
       </c>
       <c r="F50" t="n">
-        <v>1.51</v>
+        <v>1.68</v>
       </c>
       <c r="G50" t="n">
-        <v>2.31</v>
+        <v>2.02</v>
       </c>
       <c r="H50" t="inlineStr">
         <is>
@@ -2029,28 +2029,28 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>21:00</t>
+          <t>19:30</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>Itabirito (W) vs Cruzeiro (K)</t>
+          <t>Hapoel Migdal Haemeq vs Hapoel Nof HaGalil</t>
         </is>
       </c>
       <c r="C51" t="n">
-        <v>6</v>
+        <v>2.8</v>
       </c>
       <c r="D51" t="n">
-        <v>4.33</v>
+        <v>3.2</v>
       </c>
       <c r="E51" t="n">
-        <v>1.38</v>
+        <v>2.23</v>
       </c>
       <c r="F51" t="n">
-        <v>1.55</v>
+        <v>1.9</v>
       </c>
       <c r="G51" t="n">
-        <v>2.23</v>
+        <v>1.78</v>
       </c>
       <c r="H51" t="inlineStr">
         <is>
@@ -2061,28 +2061,28 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>21:00</t>
+          <t>20:00</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>Perolas Negras U20 vs Audax Rio RJ U20</t>
+          <t>MS Shikun Hamizrah vs Bnei Eilat</t>
         </is>
       </c>
       <c r="C52" t="n">
-        <v>2.04</v>
+        <v>2.39</v>
       </c>
       <c r="D52" t="n">
-        <v>3.1</v>
+        <v>3.5</v>
       </c>
       <c r="E52" t="n">
-        <v>3.2</v>
+        <v>2.36</v>
       </c>
       <c r="F52" t="n">
-        <v>2.16</v>
+        <v>1.55</v>
       </c>
       <c r="G52" t="n">
-        <v>1.58</v>
+        <v>2.25</v>
       </c>
       <c r="H52" t="inlineStr">
         <is>
@@ -2093,28 +2093,28 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>21:00</t>
+          <t>14:00</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>Sao Goncalo U20 vs Olaria RJ U20</t>
+          <t>Hapoel Bney Jdaide vs Maccabi Ihud Bnei Avtin</t>
         </is>
       </c>
       <c r="C53" t="n">
-        <v>2.55</v>
+        <v>3.15</v>
       </c>
       <c r="D53" t="n">
-        <v>3.15</v>
+        <v>3.7</v>
       </c>
       <c r="E53" t="n">
-        <v>2.4</v>
+        <v>1.87</v>
       </c>
       <c r="F53" t="n">
-        <v>1.98</v>
+        <v>1.5</v>
       </c>
       <c r="G53" t="n">
-        <v>1.71</v>
+        <v>2.37</v>
       </c>
       <c r="H53" t="inlineStr">
         <is>
@@ -2125,28 +2125,28 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>21:00</t>
+          <t>14:30</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>Sao Domingos U20 vs ASA (Agremiação Sportiva Arapiraquense) U20</t>
+          <t>Hapoel Bnei Ein Mahel vs Maccabi Maghar</t>
         </is>
       </c>
       <c r="C54" t="n">
-        <v>13.25</v>
+        <v>1.95</v>
       </c>
       <c r="D54" t="n">
-        <v>6</v>
+        <v>3.8</v>
       </c>
       <c r="E54" t="n">
-        <v>1.11</v>
+        <v>2.8</v>
       </c>
       <c r="F54" t="n">
-        <v>1.51</v>
+        <v>1.33</v>
       </c>
       <c r="G54" t="n">
-        <v>2.27</v>
+        <v>3</v>
       </c>
       <c r="H54" t="inlineStr">
         <is>
@@ -2157,28 +2157,28 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>21:00</t>
+          <t>15:30</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>Independente Atalaia U20 vs CS Esportiva U20</t>
+          <t>Maccabi Isfiya vs Hapoel Givat Olga</t>
         </is>
       </c>
       <c r="C55" t="n">
-        <v>6.5</v>
+        <v>1.96</v>
       </c>
       <c r="D55" t="n">
-        <v>4.33</v>
+        <v>3.7</v>
       </c>
       <c r="E55" t="n">
-        <v>1.33</v>
+        <v>3</v>
       </c>
       <c r="F55" t="n">
-        <v>1.6</v>
+        <v>1.41</v>
       </c>
       <c r="G55" t="n">
-        <v>2.09</v>
+        <v>2.55</v>
       </c>
       <c r="H55" t="inlineStr">
         <is>
@@ -2189,28 +2189,28 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>20:45</t>
+          <t>18:30</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>Madureira RJ vs Sampaio Correa RJ</t>
+          <t>MK Tzofi Haifa vs Tzeirey Haifa SC</t>
         </is>
       </c>
       <c r="C56" t="n">
+        <v>2.7</v>
+      </c>
+      <c r="D56" t="n">
+        <v>3.6</v>
+      </c>
+      <c r="E56" t="n">
+        <v>2.11</v>
+      </c>
+      <c r="F56" t="n">
+        <v>1.47</v>
+      </c>
+      <c r="G56" t="n">
         <v>2.45</v>
-      </c>
-      <c r="D56" t="n">
-        <v>2.9</v>
-      </c>
-      <c r="E56" t="n">
-        <v>2.68</v>
-      </c>
-      <c r="F56" t="n">
-        <v>2.37</v>
-      </c>
-      <c r="G56" t="n">
-        <v>1.5</v>
       </c>
       <c r="H56" t="inlineStr">
         <is>
@@ -2221,28 +2221,28 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>21:00</t>
+          <t>20:30</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>Gramadense RS vs EC Pelotas</t>
+          <t>Ihud Bnei Baqa vs Hapoel Bnei Arrara Ara</t>
         </is>
       </c>
       <c r="C57" t="n">
-        <v>2.37</v>
+        <v>1.37</v>
       </c>
       <c r="D57" t="n">
-        <v>2.77</v>
+        <v>4.33</v>
       </c>
       <c r="E57" t="n">
-        <v>2.9</v>
+        <v>5.5</v>
       </c>
       <c r="F57" t="n">
-        <v>2.73</v>
+        <v>1.41</v>
       </c>
       <c r="G57" t="n">
-        <v>1.38</v>
+        <v>1.53</v>
       </c>
       <c r="H57" t="inlineStr">
         <is>
@@ -2253,28 +2253,28 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>21:00</t>
+          <t>20:45</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>Gremio Esportivo Brasil RS vs Ge Gloria</t>
+          <t>Beitar Haifa Yakov vs FC Kababir</t>
         </is>
       </c>
       <c r="C58" t="n">
-        <v>1.57</v>
+        <v>1.14</v>
       </c>
       <c r="D58" t="n">
-        <v>3.4</v>
+        <v>6.5</v>
       </c>
       <c r="E58" t="n">
-        <v>5.5</v>
+        <v>11</v>
       </c>
       <c r="F58" t="n">
-        <v>2.33</v>
+        <v>1.25</v>
       </c>
       <c r="G58" t="n">
-        <v>1.51</v>
+        <v>3.5</v>
       </c>
       <c r="H58" t="inlineStr">
         <is>
@@ -2285,28 +2285,28 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>21:30</t>
+          <t>21:00</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>Esmac PA vs Pedreira EC</t>
+          <t>Maccabi Ironi Kfar Yona vs Hapoel Ramot Menashe</t>
         </is>
       </c>
       <c r="C59" t="n">
-        <v>23</v>
+        <v>1.7</v>
       </c>
       <c r="D59" t="n">
-        <v>9.5</v>
+        <v>3.8</v>
       </c>
       <c r="E59" t="n">
-        <v>1.02</v>
+        <v>3.6</v>
       </c>
       <c r="F59" t="n">
-        <v>1.16</v>
+        <v>1.43</v>
       </c>
       <c r="G59" t="n">
-        <v>4.33</v>
+        <v>2.55</v>
       </c>
       <c r="H59" t="inlineStr">
         <is>
@@ -2317,28 +2317,28 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>21:00</t>
+          <t>16:30</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>AD Confianca SE U20 vs Aracaju SE U20</t>
+          <t>Hapoel Tel Aviv (W) vs Hapoel Raanana (W)</t>
         </is>
       </c>
       <c r="C60" t="n">
-        <v>1.96</v>
+        <v>2.55</v>
       </c>
       <c r="D60" t="n">
-        <v>3.2</v>
+        <v>3.5</v>
       </c>
       <c r="E60" t="n">
-        <v>3.28</v>
+        <v>2.23</v>
       </c>
       <c r="F60" t="n">
-        <v>1.97</v>
+        <v>1.55</v>
       </c>
       <c r="G60" t="n">
-        <v>1.74</v>
+        <v>2.27</v>
       </c>
       <c r="H60" t="inlineStr">
         <is>
@@ -2349,28 +2349,28 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>21:00</t>
+          <t>16:30</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>Falcon SE U20 vs AA Guarany SE U20</t>
+          <t>Maccabi Kishronot Hadera (W) vs Maccabi Holon (W)</t>
         </is>
       </c>
       <c r="C61" t="n">
-        <v>1.32</v>
+        <v>1.57</v>
       </c>
       <c r="D61" t="n">
-        <v>5</v>
+        <v>3.8</v>
       </c>
       <c r="E61" t="n">
-        <v>6.5</v>
+        <v>4.33</v>
       </c>
       <c r="F61" t="n">
-        <v>1.32</v>
+        <v>1.47</v>
       </c>
       <c r="G61" t="n">
-        <v>3.05</v>
+        <v>2.4</v>
       </c>
       <c r="H61" t="inlineStr">
         <is>
@@ -2381,28 +2381,28 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>21:00</t>
+          <t>16:30</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>GE Prudente U20 vs CA Juventus SP U20</t>
+          <t>Hapoel Jerusalem (K) vs Kiryat Gat SC (W)</t>
         </is>
       </c>
       <c r="C62" t="n">
-        <v>2.8</v>
+        <v>2.16</v>
       </c>
       <c r="D62" t="n">
-        <v>3.3</v>
+        <v>3.5</v>
       </c>
       <c r="E62" t="n">
-        <v>2.11</v>
+        <v>2.68</v>
       </c>
       <c r="F62" t="n">
-        <v>1.78</v>
+        <v>1.57</v>
       </c>
       <c r="G62" t="n">
-        <v>1.9</v>
+        <v>2.23</v>
       </c>
       <c r="H62" t="inlineStr">
         <is>
@@ -2413,28 +2413,28 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>23:00</t>
+          <t>21:15</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>Universidad O&amp;M FC vs Atlantico Puerto Plata FC</t>
+          <t>Ik Kongahalla vs Lindome GIF</t>
         </is>
       </c>
       <c r="C63" t="n">
-        <v>1.5</v>
+        <v>2.34</v>
       </c>
       <c r="D63" t="n">
-        <v>4.33</v>
+        <v>3.7</v>
       </c>
       <c r="E63" t="n">
-        <v>4.33</v>
+        <v>2.34</v>
       </c>
       <c r="F63" t="n">
-        <v>1.25</v>
+        <v>1.32</v>
       </c>
       <c r="G63" t="n">
-        <v>3.3</v>
+        <v>2.9</v>
       </c>
       <c r="H63" t="inlineStr">
         <is>
@@ -2445,28 +2445,28 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>23:00</t>
+          <t>21:15</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>Salcedo FC vs Cibao FC</t>
+          <t>FC Bole vs FC Champagne Sport</t>
         </is>
       </c>
       <c r="C64" t="n">
-        <v>2.9</v>
+        <v>3.2</v>
       </c>
       <c r="D64" t="n">
-        <v>3.05</v>
+        <v>3.6</v>
       </c>
       <c r="E64" t="n">
-        <v>2.18</v>
+        <v>1.87</v>
       </c>
       <c r="F64" t="n">
-        <v>2.14</v>
+        <v>1.55</v>
       </c>
       <c r="G64" t="n">
-        <v>1.6</v>
+        <v>2.25</v>
       </c>
       <c r="H64" t="inlineStr">
         <is>
@@ -2477,28 +2477,28 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>32 dk içinde</t>
+          <t>21:15</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>Kuzey Kore U20 (K) vs Kolombiya U20 (K)</t>
+          <t>FC Saint-Blaise vs FC Bosna Neuchatel</t>
         </is>
       </c>
       <c r="C65" t="n">
-        <v>1.07</v>
+        <v>3.6</v>
       </c>
       <c r="D65" t="n">
-        <v>8</v>
+        <v>3.7</v>
       </c>
       <c r="E65" t="n">
-        <v>23</v>
+        <v>1.75</v>
       </c>
       <c r="F65" t="n">
-        <v>1.47</v>
+        <v>1.53</v>
       </c>
       <c r="G65" t="n">
-        <v>2.39</v>
+        <v>2.27</v>
       </c>
       <c r="H65" t="inlineStr">
         <is>
@@ -2509,29 +2509,25 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>2 dk içinde</t>
+          <t>16:45</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>SC Wiedenbruck vs VfL Osnabruck</t>
+          <t>AL Gharafa U20 vs Al-Khor U20</t>
         </is>
       </c>
       <c r="C66" t="n">
-        <v>8.5</v>
+        <v>1.45</v>
       </c>
       <c r="D66" t="n">
-        <v>5.5</v>
+        <v>4</v>
       </c>
       <c r="E66" t="n">
-        <v>1.22</v>
-      </c>
-      <c r="F66" t="n">
-        <v>1.3</v>
-      </c>
-      <c r="G66" t="n">
-        <v>3.15</v>
-      </c>
+        <v>6</v>
+      </c>
+      <c r="F66" t="inlineStr"/>
+      <c r="G66" t="inlineStr"/>
       <c r="H66" t="inlineStr">
         <is>
           <t>-</t>
@@ -2541,28 +2537,28 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>21:00</t>
+          <t>16:45</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>West Ham U21 vs Valencia U21</t>
+          <t>Umm Salal U20 vs Al-Markhiya U20</t>
         </is>
       </c>
       <c r="C67" t="n">
-        <v>2.27</v>
+        <v>2.1</v>
       </c>
       <c r="D67" t="n">
         <v>3.5</v>
       </c>
       <c r="E67" t="n">
-        <v>2.5</v>
+        <v>2.7</v>
       </c>
       <c r="F67" t="n">
-        <v>1.53</v>
+        <v>1.51</v>
       </c>
       <c r="G67" t="n">
-        <v>2.3</v>
+        <v>2.26</v>
       </c>
       <c r="H67" t="inlineStr">
         <is>
@@ -2573,28 +2569,28 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>21:00</t>
+          <t>17:45</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>Middlesbrough U21 vs KRC Genk U21</t>
+          <t>Al Sadd U20 vs Mesaimeer U20</t>
         </is>
       </c>
       <c r="C68" t="n">
-        <v>2.8</v>
+        <v>1.76</v>
       </c>
       <c r="D68" t="n">
-        <v>3.7</v>
+        <v>4</v>
       </c>
       <c r="E68" t="n">
-        <v>1.97</v>
+        <v>3.4</v>
       </c>
       <c r="F68" t="n">
-        <v>1.41</v>
+        <v>1.51</v>
       </c>
       <c r="G68" t="n">
-        <v>2.63</v>
+        <v>2.26</v>
       </c>
       <c r="H68" t="inlineStr">
         <is>
@@ -2605,28 +2601,28 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>2 dk içinde</t>
+          <t>17:45</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>Cebelitarık vs Sao Tome and Principe</t>
+          <t>Al-Arabi Doha U20 vs Al-Duhail U20</t>
         </is>
       </c>
       <c r="C69" t="n">
-        <v>1.47</v>
+        <v>1.58</v>
       </c>
       <c r="D69" t="n">
-        <v>4.25</v>
+        <v>4</v>
       </c>
       <c r="E69" t="n">
-        <v>5.5</v>
+        <v>4.15</v>
       </c>
       <c r="F69" t="n">
-        <v>1.6</v>
+        <v>1.43</v>
       </c>
       <c r="G69" t="n">
-        <v>2.16</v>
+        <v>1.51</v>
       </c>
       <c r="H69" t="inlineStr">
         <is>
@@ -2637,28 +2633,28 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>2 dk içinde</t>
+          <t>18:55</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>Azerbaycan vs Tacikistan</t>
+          <t>Al-Wakrah U20 vs Qatar SC U20</t>
         </is>
       </c>
       <c r="C70" t="n">
-        <v>1.74</v>
+        <v>3.5</v>
       </c>
       <c r="D70" t="n">
-        <v>3.4</v>
+        <v>3.2</v>
       </c>
       <c r="E70" t="n">
-        <v>4.5</v>
+        <v>1.97</v>
       </c>
       <c r="F70" t="n">
-        <v>2.14</v>
+        <v>1.43</v>
       </c>
       <c r="G70" t="n">
-        <v>1.64</v>
+        <v>1.51</v>
       </c>
       <c r="H70" t="inlineStr">
         <is>
@@ -2669,25 +2665,29 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>2 dk içinde</t>
+          <t>22:00</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>Army Ladies FC (W) vs Epiphany Warriors (W)</t>
+          <t>Cariari Pococi vs Pitbulls Santa Barbara</t>
         </is>
       </c>
       <c r="C71" t="n">
+        <v>2.2</v>
+      </c>
+      <c r="D71" t="n">
+        <v>3.3</v>
+      </c>
+      <c r="E71" t="n">
+        <v>2.73</v>
+      </c>
+      <c r="F71" t="n">
         <v>1.72</v>
       </c>
-      <c r="D71" t="n">
-        <v>3.2</v>
-      </c>
-      <c r="E71" t="n">
-        <v>4.5</v>
-      </c>
-      <c r="F71" t="inlineStr"/>
-      <c r="G71" t="inlineStr"/>
+      <c r="G71" t="n">
+        <v>1.92</v>
+      </c>
       <c r="H71" t="inlineStr">
         <is>
           <t>-</t>
@@ -2697,25 +2697,25 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>20:00</t>
+          <t>22:00</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>Peru U19 vs Argentina U19</t>
+          <t>Porto Riko vs Guyana</t>
         </is>
       </c>
       <c r="C72" t="n">
-        <v>7</v>
+        <v>2.7</v>
       </c>
       <c r="D72" t="n">
-        <v>3.8</v>
+        <v>3.2</v>
       </c>
       <c r="E72" t="n">
-        <v>1.38</v>
+        <v>2.4</v>
       </c>
       <c r="F72" t="n">
-        <v>1.97</v>
+        <v>1.99</v>
       </c>
       <c r="G72" t="n">
         <v>1.72</v>
@@ -2729,28 +2729,28 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>23:00</t>
+          <t>16:30</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>Paraguay U19 vs Chile U19</t>
+          <t>Fk Teteks vs Rabotnicki Skopje</t>
         </is>
       </c>
       <c r="C73" t="n">
-        <v>2.1</v>
+        <v>4.2</v>
       </c>
       <c r="D73" t="n">
-        <v>3.4</v>
+        <v>3.6</v>
       </c>
       <c r="E73" t="n">
-        <v>2.9</v>
+        <v>1.64</v>
       </c>
       <c r="F73" t="n">
-        <v>1.8</v>
+        <v>1.72</v>
       </c>
       <c r="G73" t="n">
-        <v>1.93</v>
+        <v>1.95</v>
       </c>
       <c r="H73" t="inlineStr">
         <is>
@@ -2761,28 +2761,28 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>21:00</t>
+          <t>16:30</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>Chile U20 (W) vs Venezuela U20 (W)</t>
+          <t>Detonit Plackovica vs Ohrid</t>
         </is>
       </c>
       <c r="C74" t="n">
-        <v>1.74</v>
+        <v>4.5</v>
       </c>
       <c r="D74" t="n">
         <v>3.5</v>
       </c>
       <c r="E74" t="n">
-        <v>3.8</v>
+        <v>1.6</v>
       </c>
       <c r="F74" t="n">
-        <v>1.81</v>
+        <v>1.87</v>
       </c>
       <c r="G74" t="n">
-        <v>1.87</v>
+        <v>1.78</v>
       </c>
       <c r="H74" t="inlineStr">
         <is>
@@ -2793,28 +2793,28 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>21:45</t>
+          <t>16:30</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>Hamilton Academical FC vs Cowdenbeath</t>
+          <t>Mogila vs Aresimi 1973</t>
         </is>
       </c>
       <c r="C75" t="n">
-        <v>1.14</v>
+        <v>31</v>
       </c>
       <c r="D75" t="n">
-        <v>7</v>
+        <v>17</v>
       </c>
       <c r="E75" t="n">
-        <v>11</v>
+        <v>1.07</v>
       </c>
       <c r="F75" t="n">
-        <v>1.22</v>
+        <v>1.07</v>
       </c>
       <c r="G75" t="n">
-        <v>3.6</v>
+        <v>6.5</v>
       </c>
       <c r="H75" t="inlineStr">
         <is>
@@ -2825,28 +2825,28 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>21:45</t>
+          <t>18:00</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>Cumnock Juniors FC vs Troon FC</t>
+          <t>Rivers United vs Kun Khalifat FC</t>
         </is>
       </c>
       <c r="C76" t="n">
-        <v>1.8</v>
+        <v>1.22</v>
       </c>
       <c r="D76" t="n">
-        <v>3.8</v>
+        <v>5</v>
       </c>
       <c r="E76" t="n">
-        <v>3.28</v>
+        <v>8</v>
       </c>
       <c r="F76" t="n">
-        <v>1.38</v>
+        <v>1.47</v>
       </c>
       <c r="G76" t="n">
-        <v>2.73</v>
+        <v>2.37</v>
       </c>
       <c r="H76" t="inlineStr">
         <is>
@@ -2857,28 +2857,28 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>1 dk içinde</t>
+          <t>21:00</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>Ironi Beit Shemesh vs Agudat Sport Nordia Jerusalem</t>
+          <t>Grorud U19 vs Valerenga U19</t>
         </is>
       </c>
       <c r="C77" t="n">
-        <v>1.47</v>
+        <v>1.35</v>
       </c>
       <c r="D77" t="n">
-        <v>4.15</v>
+        <v>4.75</v>
       </c>
       <c r="E77" t="n">
-        <v>4.75</v>
+        <v>4.5</v>
       </c>
       <c r="F77" t="n">
-        <v>1.47</v>
+        <v>1.12</v>
       </c>
       <c r="G77" t="n">
-        <v>2.4</v>
+        <v>5</v>
       </c>
       <c r="H77" t="inlineStr">
         <is>
@@ -2889,28 +2889,28 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>1 dk içinde</t>
+          <t>21:15</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>Hapoel Marmorek vs Shimshon Tel Aviv</t>
+          <t>Haslum IL U19 vs Asker U19</t>
         </is>
       </c>
       <c r="C78" t="n">
-        <v>4.15</v>
+        <v>1.45</v>
       </c>
       <c r="D78" t="n">
-        <v>3.3</v>
+        <v>5</v>
       </c>
       <c r="E78" t="n">
-        <v>1.72</v>
+        <v>4.25</v>
       </c>
       <c r="F78" t="n">
-        <v>2.07</v>
+        <v>1.08</v>
       </c>
       <c r="G78" t="n">
-        <v>1.66</v>
+        <v>6.5</v>
       </c>
       <c r="H78" t="inlineStr">
         <is>
@@ -2921,28 +2921,28 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>20:10</t>
+          <t>21:15</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>Sport Club Dimona vs Maccabi Kiryat Malakhi</t>
+          <t>IF Ready U19 vs Skedsmo U19</t>
         </is>
       </c>
       <c r="C79" t="n">
-        <v>1.98</v>
+        <v>1.84</v>
       </c>
       <c r="D79" t="n">
-        <v>3.2</v>
+        <v>4.25</v>
       </c>
       <c r="E79" t="n">
-        <v>3.3</v>
+        <v>2.8</v>
       </c>
       <c r="F79" t="n">
-        <v>2.06</v>
+        <v>1.13</v>
       </c>
       <c r="G79" t="n">
-        <v>1.66</v>
+        <v>5</v>
       </c>
       <c r="H79" t="inlineStr">
         <is>
@@ -2953,28 +2953,28 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>20:15</t>
+          <t>21:15</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>Hapoel Ramat Hasharon vs Sderot FC</t>
+          <t>Sprint/Jeloy U19 vs Sarpsborg 08 U19</t>
         </is>
       </c>
       <c r="C80" t="n">
-        <v>1.99</v>
+        <v>1.33</v>
       </c>
       <c r="D80" t="n">
-        <v>3.3</v>
+        <v>5</v>
       </c>
       <c r="E80" t="n">
-        <v>3.1</v>
+        <v>5</v>
       </c>
       <c r="F80" t="n">
-        <v>1.8</v>
+        <v>1.14</v>
       </c>
       <c r="G80" t="n">
-        <v>1.87</v>
+        <v>4.75</v>
       </c>
       <c r="H80" t="inlineStr">
         <is>
@@ -2985,28 +2985,28 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>20:15</t>
+          <t>21:15</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>Hapoel Herzliya vs MS Tzeirey Tira</t>
+          <t>Christiania BK U19 vs Gjovik Lyn U19</t>
         </is>
       </c>
       <c r="C81" t="n">
-        <v>1.85</v>
+        <v>1.03</v>
       </c>
       <c r="D81" t="n">
-        <v>3.2</v>
+        <v>10</v>
       </c>
       <c r="E81" t="n">
-        <v>3.6</v>
+        <v>34</v>
       </c>
       <c r="F81" t="n">
-        <v>2.06</v>
+        <v>1.14</v>
       </c>
       <c r="G81" t="n">
-        <v>1.66</v>
+        <v>4.75</v>
       </c>
       <c r="H81" t="inlineStr">
         <is>
@@ -3017,28 +3017,28 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>20:00</t>
+          <t>21:15</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>Sport Club Tira vs Hapoel Bnei Musmus</t>
+          <t>Baerum Sk U19 vs Ullern U19</t>
         </is>
       </c>
       <c r="C82" t="n">
-        <v>1.58</v>
+        <v>2.12</v>
       </c>
       <c r="D82" t="n">
-        <v>3.7</v>
+        <v>4.25</v>
       </c>
       <c r="E82" t="n">
-        <v>4.5</v>
+        <v>2.37</v>
       </c>
       <c r="F82" t="n">
-        <v>1.71</v>
+        <v>1.1</v>
       </c>
       <c r="G82" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="H82" t="inlineStr">
         <is>
@@ -3049,28 +3049,28 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>20:00</t>
+          <t>21:15</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>Beitar Naharia vs Maccabi Neve Shaanan Eldad</t>
+          <t>KFUM U19 vs Nordstrand U19</t>
         </is>
       </c>
       <c r="C83" t="n">
-        <v>1.81</v>
+        <v>1.2</v>
       </c>
       <c r="D83" t="n">
-        <v>3.4</v>
+        <v>5.5</v>
       </c>
       <c r="E83" t="n">
-        <v>3.6</v>
+        <v>6.5</v>
       </c>
       <c r="F83" t="n">
-        <v>1.85</v>
+        <v>1.09</v>
       </c>
       <c r="G83" t="n">
-        <v>1.83</v>
+        <v>5.5</v>
       </c>
       <c r="H83" t="inlineStr">
         <is>
@@ -3081,28 +3081,28 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>20:20</t>
+          <t>21:15</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>Tzeirei Umm al-Fahm vs Hapoel Umm Al Fahm</t>
+          <t>Follo U19 vs Lillehammer U19</t>
         </is>
       </c>
       <c r="C84" t="n">
-        <v>4.15</v>
+        <v>1.55</v>
       </c>
       <c r="D84" t="n">
-        <v>3.8</v>
+        <v>4.25</v>
       </c>
       <c r="E84" t="n">
-        <v>1.6</v>
+        <v>3.3</v>
       </c>
       <c r="F84" t="n">
-        <v>1.55</v>
+        <v>1.12</v>
       </c>
       <c r="G84" t="n">
-        <v>2.23</v>
+        <v>5</v>
       </c>
       <c r="H84" t="inlineStr">
         <is>
@@ -3113,28 +3113,28 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>20:45</t>
+          <t>21:30</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>Hapoel Ironi Baqa Al-Gharbiyye vs Hapoel Tirat HaCarmel</t>
+          <t>Raelingen U19 vs Gjelleraasen U19</t>
         </is>
       </c>
       <c r="C85" t="n">
-        <v>1.78</v>
+        <v>23</v>
       </c>
       <c r="D85" t="n">
-        <v>3.5</v>
+        <v>9</v>
       </c>
       <c r="E85" t="n">
-        <v>3.5</v>
+        <v>1.05</v>
       </c>
       <c r="F85" t="n">
-        <v>1.64</v>
+        <v>1.12</v>
       </c>
       <c r="G85" t="n">
-        <v>2.07</v>
+        <v>5</v>
       </c>
       <c r="H85" t="inlineStr">
         <is>
@@ -3145,28 +3145,28 @@
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>21:15</t>
+          <t>21:30</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>Hapoel Bnei Lod vs Beitar Tel Aviv Holon</t>
+          <t>Lorenskog U19 vs Kjelsas U19</t>
         </is>
       </c>
       <c r="C86" t="n">
-        <v>1.62</v>
+        <v>5</v>
       </c>
       <c r="D86" t="n">
-        <v>3.8</v>
+        <v>5</v>
       </c>
       <c r="E86" t="n">
-        <v>4.2</v>
+        <v>1.3</v>
       </c>
       <c r="F86" t="n">
-        <v>1.87</v>
+        <v>1.14</v>
       </c>
       <c r="G86" t="n">
-        <v>1.79</v>
+        <v>4.75</v>
       </c>
       <c r="H86" t="inlineStr">
         <is>
@@ -3177,28 +3177,28 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>1 dk içinde</t>
+          <t>17:30</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>Sandvikens IF (W) vs Umea IK (W)</t>
+          <t>Oman Club vs Sur Club</t>
         </is>
       </c>
       <c r="C87" t="n">
-        <v>4.2</v>
+        <v>3.8</v>
       </c>
       <c r="D87" t="n">
-        <v>4</v>
+        <v>3.2</v>
       </c>
       <c r="E87" t="n">
+        <v>1.81</v>
+      </c>
+      <c r="F87" t="n">
+        <v>2.18</v>
+      </c>
+      <c r="G87" t="n">
         <v>1.58</v>
-      </c>
-      <c r="F87" t="n">
-        <v>1.6</v>
-      </c>
-      <c r="G87" t="n">
-        <v>2.07</v>
       </c>
       <c r="H87" t="inlineStr">
         <is>
@@ -3209,28 +3209,28 @@
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>21:00</t>
+          <t>17:40</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>FC Haute-Ajoie vs FC Ajoie-Monterri</t>
+          <t>Sohar Club vs Al Seeb</t>
         </is>
       </c>
       <c r="C88" t="n">
-        <v>2.2</v>
+        <v>2.23</v>
       </c>
       <c r="D88" t="n">
-        <v>3.5</v>
+        <v>3.05</v>
       </c>
       <c r="E88" t="n">
-        <v>2.68</v>
+        <v>2.9</v>
       </c>
       <c r="F88" t="n">
-        <v>1.57</v>
+        <v>2.18</v>
       </c>
       <c r="G88" t="n">
-        <v>2.25</v>
+        <v>1.58</v>
       </c>
       <c r="H88" t="inlineStr">
         <is>
@@ -3241,28 +3241,28 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>22:00</t>
+          <t>16:30</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>Turks and Caicos Islands vs Montserrat</t>
+          <t>FK Podkonice vs MFK Ruzomberok B</t>
         </is>
       </c>
       <c r="C89" t="n">
-        <v>12</v>
+        <v>2.58</v>
       </c>
       <c r="D89" t="n">
-        <v>6.5</v>
+        <v>3.3</v>
       </c>
       <c r="E89" t="n">
-        <v>1.16</v>
+        <v>2.31</v>
       </c>
       <c r="F89" t="n">
-        <v>1.4</v>
+        <v>1.74</v>
       </c>
       <c r="G89" t="n">
-        <v>2.7</v>
+        <v>1.96</v>
       </c>
       <c r="H89" t="inlineStr">
         <is>
@@ -3273,28 +3273,28 @@
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>23:00</t>
+          <t>21:30</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>Bahamas vs Saint Martin</t>
+          <t>Montevideo City Torque vs Atenas</t>
         </is>
       </c>
       <c r="C90" t="n">
-        <v>15</v>
+        <v>1.53</v>
       </c>
       <c r="D90" t="n">
-        <v>7.5</v>
+        <v>3.7</v>
       </c>
       <c r="E90" t="n">
-        <v>1.12</v>
+        <v>5</v>
       </c>
       <c r="F90" t="n">
-        <v>1.32</v>
+        <v>1.79</v>
       </c>
       <c r="G90" t="n">
-        <v>3.05</v>
+        <v>1.87</v>
       </c>
       <c r="H90" t="inlineStr">
         <is>
@@ -3305,28 +3305,28 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>59 dk içinde</t>
+          <t>21:30</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>Necaxa U21 vs Atletico San Luis U21</t>
+          <t>Danubio vs Penarol Montevideo</t>
         </is>
       </c>
       <c r="C91" t="n">
-        <v>1.95</v>
+        <v>3.3</v>
       </c>
       <c r="D91" t="n">
-        <v>3.8</v>
+        <v>3.05</v>
       </c>
       <c r="E91" t="n">
-        <v>2.9</v>
+        <v>2.05</v>
       </c>
       <c r="F91" t="n">
-        <v>1.37</v>
+        <v>2.27</v>
       </c>
       <c r="G91" t="n">
-        <v>2.8</v>
+        <v>1.53</v>
       </c>
       <c r="H91" t="inlineStr">
         <is>
@@ -3337,28 +3337,28 @@
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>21:00</t>
+          <t>19:00</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>Tlapa Mazatecochco vs Dragones de Oaxaca II</t>
+          <t>AL Ahli Amman vs Ma'an</t>
         </is>
       </c>
       <c r="C92" t="n">
-        <v>2.1</v>
+        <v>1.66</v>
       </c>
       <c r="D92" t="n">
-        <v>3.4</v>
+        <v>3.5</v>
       </c>
       <c r="E92" t="n">
-        <v>2.77</v>
+        <v>4.2</v>
       </c>
       <c r="F92" t="n">
-        <v>1.58</v>
+        <v>1.81</v>
       </c>
       <c r="G92" t="n">
-        <v>2.12</v>
+        <v>1.86</v>
       </c>
       <c r="H92" t="inlineStr">
         <is>
@@ -3369,28 +3369,28 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>22:00</t>
+          <t>19:00</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>Artesanos Metepec FC vs Toluca U21</t>
+          <t>Sahl Horan SC vs Hayy Al-Amir Hassan</t>
         </is>
       </c>
       <c r="C93" t="n">
-        <v>2.45</v>
+        <v>2.2</v>
       </c>
       <c r="D93" t="n">
-        <v>3.4</v>
+        <v>3</v>
       </c>
       <c r="E93" t="n">
-        <v>2.45</v>
+        <v>2.9</v>
       </c>
       <c r="F93" t="n">
-        <v>1.72</v>
+        <v>2.22</v>
       </c>
       <c r="G93" t="n">
-        <v>1.93</v>
+        <v>1.55</v>
       </c>
       <c r="H93" t="inlineStr">
         <is>
@@ -3401,28 +3401,28 @@
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>22:00</t>
+          <t>19:00</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>Sportivo San Lorenzo vs 4 de Mayo</t>
+          <t>Nashama Al-Mustaqbal (W) vs Al Orthodoxi (W)</t>
         </is>
       </c>
       <c r="C94" t="n">
-        <v>1.11</v>
+        <v>2.04</v>
       </c>
       <c r="D94" t="n">
-        <v>7.5</v>
+        <v>3.5</v>
       </c>
       <c r="E94" t="n">
-        <v>15</v>
+        <v>2.8</v>
       </c>
       <c r="F94" t="n">
-        <v>1.38</v>
+        <v>1.58</v>
       </c>
       <c r="G94" t="n">
-        <v>2.73</v>
+        <v>2.2</v>
       </c>
       <c r="H94" t="inlineStr">
         <is>
@@ -3433,94 +3433,30 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>23:00</t>
+          <t>16:00</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>Asociacion Deportiva Tarma vs Cienciano Cusco</t>
+          <t>Uhamiaji FC vs Raskazone</t>
         </is>
       </c>
       <c r="C95" t="n">
-        <v>2.9</v>
+        <v>1.5</v>
       </c>
       <c r="D95" t="n">
-        <v>3.5</v>
+        <v>3.7</v>
       </c>
       <c r="E95" t="n">
-        <v>2.11</v>
+        <v>5.5</v>
       </c>
       <c r="F95" t="n">
-        <v>1.66</v>
+        <v>1.96</v>
       </c>
       <c r="G95" t="n">
-        <v>2.08</v>
+        <v>1.72</v>
       </c>
       <c r="H95" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-    </row>
-    <row r="96">
-      <c r="A96" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="B96" t="inlineStr">
-        <is>
-          <t>Boston River vs Centro Atletico Fenix Montevideo</t>
-        </is>
-      </c>
-      <c r="C96" t="n">
-        <v>2.01</v>
-      </c>
-      <c r="D96" t="n">
-        <v>3.1</v>
-      </c>
-      <c r="E96" t="n">
-        <v>3.3</v>
-      </c>
-      <c r="F96" t="n">
-        <v>2.15</v>
-      </c>
-      <c r="G96" t="n">
-        <v>1.6</v>
-      </c>
-      <c r="H96" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-    </row>
-    <row r="97">
-      <c r="A97" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="B97" t="inlineStr">
-        <is>
-          <t>Liverpool Montevideo vs Colon FC</t>
-        </is>
-      </c>
-      <c r="C97" t="n">
-        <v>1.5</v>
-      </c>
-      <c r="D97" t="n">
-        <v>3.7</v>
-      </c>
-      <c r="E97" t="n">
-        <v>5.5</v>
-      </c>
-      <c r="F97" t="n">
-        <v>1.98</v>
-      </c>
-      <c r="G97" t="n">
-        <v>1.72</v>
-      </c>
-      <c r="H97" t="inlineStr">
         <is>
           <t>-</t>
         </is>

</xml_diff>